<commit_message>
Project BugReproducing is saved.
</commit_message>
<xml_diff>
--- a/EEEEE/BugReproducing/BugReproducing.xlsx
+++ b/EEEEE/BugReproducing/BugReproducing.xlsx
@@ -14,6 +14,7 @@
   </bookViews>
   <sheets>
     <sheet name="Alg" sheetId="4" r:id="rId1"/>
+    <sheet name="calc1" r:id="rId5" sheetId="5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="54">
   <si>
     <t>Step</t>
   </si>
@@ -163,6 +164,39 @@
   </si>
   <si>
     <t>= calc2 (originalValue.someValue[0], overriddenValuess.someValue)</t>
+  </si>
+  <si>
+    <t>Test calc1 calc1Test</t>
+  </si>
+  <si>
+    <t>originalValue.a</t>
+  </si>
+  <si>
+    <t>_res_</t>
+  </si>
+  <si>
+    <t>Original Value A</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>result_id_1</t>
+  </si>
+  <si>
+    <t>_res_.$Step1</t>
+  </si>
+  <si>
+    <t>Test calc2 calc1Test</t>
+  </si>
+  <si>
+    <t>someInputValue.a</t>
+  </si>
+  <si>
+    <t>_res_.$OverriddenType1</t>
   </si>
 </sst>
 </file>
@@ -173,7 +207,7 @@
   <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="1" rgb="000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -963,4 +997,45 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="B2:C5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="0"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C5" s="0"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>